<commit_message>
Save the complete version 1 on Feb 15.
</commit_message>
<xml_diff>
--- a/results/tables/01_contamination_assessment/table1_pca_loadings.xlsx
+++ b/results/tables/01_contamination_assessment/table1_pca_loadings.xlsx
@@ -425,15 +425,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>var</t>
-        </is>
-      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>PC1</t>
@@ -468,751 +463,485 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>%OC</t>
+          <t>Co</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.2397725329432298</v>
+        <v>0.3606101831871588</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0102375511536948</v>
+        <v>0.1877290339865944</v>
       </c>
       <c r="D2" t="n">
-        <v>-0.06193854944746077</v>
+        <v>0.1119599705742961</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1266510966322322</v>
+        <v>0.3202135299974001</v>
       </c>
       <c r="F2" t="n">
-        <v>0.001672147967784248</v>
+        <v>-0.06073174242921327</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.02742863127172494</v>
+        <v>0.05937564749851851</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>1234-TCB</t>
+          <t>Al</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.06150624875934518</v>
+        <v>0.5214695814339583</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.0145577220325552</v>
+        <v>0.1832330240339628</v>
       </c>
       <c r="D3" t="n">
-        <v>0.04926358724710705</v>
+        <v>0.3068722930964033</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2243516196629816</v>
+        <v>0.7292323415583598</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1143782919208221</v>
+        <v>-0.05202754895816125</v>
       </c>
       <c r="G3" t="n">
-        <v>0.7923563674208387</v>
+        <v>0.1492353506633274</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>1245-TCB</t>
+          <t>Ni</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.104572328105209</v>
+        <v>0.4094264607169094</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3571725802913596</v>
+        <v>0.9272058070250112</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0924180711471228</v>
+        <v>-0.04979837077098496</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.2376245554450821</v>
+        <v>0.2056390972923768</v>
       </c>
       <c r="F4" t="n">
-        <v>0.02230957672424659</v>
+        <v>-0.2132220398666368</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.03112850058895784</v>
+        <v>0.002759796000171527</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Al</t>
+          <t>Mn</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.2492388211887576</v>
+        <v>0.06507095861101514</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.02934657894629875</v>
+        <v>0.2746698837258384</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.1889796293267045</v>
+        <v>0.3508990558530958</v>
       </c>
       <c r="E5" t="n">
-        <v>0.03991761245108588</v>
+        <v>0.3814571777589376</v>
       </c>
       <c r="F5" t="n">
-        <v>0.1703236209212356</v>
+        <v>0.06571909405534154</v>
       </c>
       <c r="G5" t="n">
-        <v>-0.1192847667729189</v>
+        <v>0.1675764027806538</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>As</t>
+          <t>Fe</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1423631461075968</v>
+        <v>0.5073370775090991</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.1518719711138822</v>
+        <v>0.3433756328793434</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.0708138340069272</v>
+        <v>0.1304823760386074</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.2066481029457917</v>
+        <v>0.6099595439975646</v>
       </c>
       <c r="F6" t="n">
-        <v>0.08943470558294155</v>
+        <v>0.7153959372751683</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.04517247399399055</v>
+        <v>-0.4865255919213472</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Bi</t>
+          <t>Cr</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-0.09945288642347773</v>
+        <v>0.6719704293106613</v>
       </c>
       <c r="C7" t="n">
-        <v>0.2881793704444597</v>
+        <v>0.5670885411507882</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.03072170173970704</v>
+        <v>0.106670535502527</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3977917895819559</v>
+        <v>0.3577982473586992</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.01632984691249517</v>
+        <v>-0.2422077762230097</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.1472542939704907</v>
+        <v>-0.04704343808838031</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Ca</t>
+          <t>Cu</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1488615737826672</v>
+        <v>0.7543749497540863</v>
       </c>
       <c r="C8" t="n">
-        <v>0.2410124046548661</v>
+        <v>0.6971553913821574</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.09241130733865702</v>
+        <v>0.1474068558952266</v>
       </c>
       <c r="E8" t="n">
-        <v>0.2841640342603037</v>
+        <v>0.4925226869386944</v>
       </c>
       <c r="F8" t="n">
-        <v>0.01878993921553548</v>
+        <v>-0.4369477504943916</v>
       </c>
       <c r="G8" t="n">
-        <v>0.06507785872199459</v>
+        <v>-0.0759409071495515</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Cd</t>
+          <t>Hg</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.1345116606250814</v>
+        <v>5.107143789904225</v>
       </c>
       <c r="C9" t="n">
-        <v>0.1452662109119351</v>
+        <v>-0.6096427455103576</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2955964866302596</v>
+        <v>0.07425475450888282</v>
       </c>
       <c r="E9" t="n">
-        <v>0.2916259129278473</v>
+        <v>0.183992574608914</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.2261518509066956</v>
+        <v>-0.01137937574588698</v>
       </c>
       <c r="G9" t="n">
-        <v>0.03481477075560681</v>
+        <v>0.03154523788975458</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Co</t>
+          <t>Pb</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.2530332524743897</v>
+        <v>-0.1038857224785213</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.02801197978054151</v>
+        <v>0.4042564135127725</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.1276068437611494</v>
+        <v>1.473122055190723</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.03688391138056726</v>
+        <v>-0.4778803022358065</v>
       </c>
       <c r="F10" t="n">
-        <v>0.1392992442451483</v>
+        <v>0.02409371635469992</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.08627179012996071</v>
+        <v>-0.01518205199926889</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Cr</t>
+          <t>Zn</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.2550769640276756</v>
+        <v>-2.335244129682883</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.1151907001018954</v>
+        <v>0.7543773998348152</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0485621926465865</v>
+        <v>0.2227753496080398</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.01234035803666223</v>
+        <v>0.4044778329318201</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.147184827680691</v>
+        <v>0.01610606886892633</v>
       </c>
       <c r="G11" t="n">
-        <v>0.01054492300817206</v>
+        <v>0.01916492083667855</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
-          <t>Cu</t>
+          <t>total PCB</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.2290453142952631</v>
+        <v>1.682317074569096</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.1514063909095279</v>
+        <v>1.711686459665509</v>
       </c>
       <c r="D12" t="n">
-        <v>0.01887509588829825</v>
+        <v>-0.5485684584588472</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.04010273173193573</v>
+        <v>-0.7048118292085341</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.2512990936678288</v>
+        <v>0.1614578467457171</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.04272685959379767</v>
+        <v>0.001747225344804268</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
         <is>
-          <t>Fe</t>
+          <t>Cd</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.2550559173010482</v>
+        <v>0.3997005489335929</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.05115316586065696</v>
+        <v>0.2211779878078544</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.09144854493810042</v>
+        <v>0.1854150206582691</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.1007314459410343</v>
+        <v>-0.06578916343869991</v>
       </c>
       <c r="F13" t="n">
-        <v>0.1470730845207363</v>
+        <v>-0.04718811875168219</v>
       </c>
       <c r="G13" t="n">
-        <v>0.1436710283507441</v>
+        <v>0.008309499005907571</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
         <is>
-          <t>HCB</t>
+          <t>OCS</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.06626983023537687</v>
+        <v>0.03956333063927631</v>
       </c>
       <c r="C14" t="n">
-        <v>0.3687388847232415</v>
+        <v>0.1869113238801454</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1067956232109586</v>
+        <v>-0.03677150855389216</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.2044526351841423</v>
+        <v>0.05473297279913972</v>
       </c>
       <c r="F14" t="n">
-        <v>0.1814640999109</v>
+        <v>0.3936352260306018</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1606353226722459</v>
+        <v>0.6206645199379749</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
         <is>
-          <t>Heptachlor Epoxide</t>
+          <t>p,p'-DDE</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-0.03891903504286543</v>
+        <v>0.6317417252198432</v>
       </c>
       <c r="C15" t="n">
-        <v>0.03300613399993117</v>
+        <v>0.5112024472909085</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2034534428703216</v>
+        <v>-0.2180187387240261</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1061736848756154</v>
+        <v>-0.1479949182682809</v>
       </c>
       <c r="F15" t="n">
-        <v>0.5046911685123014</v>
+        <v>0.03411852705251382</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1615590379537958</v>
+        <v>0.05127600188288441</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
-          <t>Hg</t>
+          <t>As</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.1189236118338499</v>
+        <v>0.8038463549921078</v>
       </c>
       <c r="C16" t="n">
-        <v>0.1751174746022823</v>
+        <v>-0.04268633717272017</v>
       </c>
       <c r="D16" t="n">
-        <v>0.3562420464155425</v>
+        <v>1.01681817994705</v>
       </c>
       <c r="E16" t="n">
-        <v>0.009245042482894148</v>
+        <v>-0.3993110320221156</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.06680698161465769</v>
+        <v>0.05105283293193173</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.193724492925444</v>
+        <v>-0.008260379517027678</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
         <is>
-          <t>K</t>
+          <t>Ca</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.2390735746469758</v>
+        <v>0.1557326474084392</v>
       </c>
       <c r="C17" t="n">
-        <v>0.04283064613446903</v>
+        <v>0.07203148140934948</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.1782343150630561</v>
+        <v>0.08152911706652521</v>
       </c>
       <c r="E17" t="n">
-        <v>0.1383646696543311</v>
+        <v>0.3426865634316861</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1740049195747403</v>
+        <v>0.1848546464642934</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.1253238102224767</v>
+        <v>0.3208503623931828</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Mg</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>0.170578192755395</v>
-      </c>
-      <c r="C18" t="n">
-        <v>0.2160357517613905</v>
-      </c>
-      <c r="D18" t="n">
-        <v>-0.1355468499145729</v>
-      </c>
-      <c r="E18" t="n">
-        <v>0.2701317417426021</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0.01671826060664746</v>
-      </c>
-      <c r="G18" t="n">
-        <v>-0.05690496018811007</v>
-      </c>
+      <c r="A18" s="1" t="inlineStr"/>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
         <is>
-          <t>Mn</t>
+          <t>Explained Variance</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.2497658776084371</v>
+        <v>37.45996204980186</v>
       </c>
       <c r="C19" t="n">
-        <v>0.01800195900650422</v>
+        <v>6.31573003109829</v>
       </c>
       <c r="D19" t="n">
-        <v>-0.1642631864428569</v>
+        <v>3.932436519405018</v>
       </c>
       <c r="E19" t="n">
-        <v>0.102306075482773</v>
+        <v>2.793457029766627</v>
       </c>
       <c r="F19" t="n">
-        <v>0.05451660709676741</v>
+        <v>1.039712293364102</v>
       </c>
       <c r="G19" t="n">
-        <v>-0.01248539292777923</v>
+        <v>0.7911052377804028</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
         <is>
-          <t>Na</t>
+          <t>Proportion of Variance</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.2224025710410987</v>
+        <v>0.6864431839375965</v>
       </c>
       <c r="C20" t="n">
-        <v>0.1312244049878352</v>
+        <v>0.115733962188046</v>
       </c>
       <c r="D20" t="n">
-        <v>-0.1279265630644192</v>
+        <v>0.0720607842961533</v>
       </c>
       <c r="E20" t="n">
-        <v>0.01263276551472529</v>
+        <v>0.05118930807128268</v>
       </c>
       <c r="F20" t="n">
-        <v>-0.06816120146863686</v>
+        <v>0.01905243299731773</v>
       </c>
       <c r="G20" t="n">
-        <v>-0.1209906620742878</v>
+        <v>0.01449677918866342</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
         <is>
-          <t>Ni</t>
+          <t>Cumulative Proportion</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.2736352158646948</v>
+        <v>0.6864431839375965</v>
       </c>
       <c r="C21" t="n">
-        <v>-0.05015740695595455</v>
+        <v>0.8021771461256425</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.01281308577408671</v>
+        <v>0.8742379304217958</v>
       </c>
       <c r="E21" t="n">
-        <v>-0.0006990812857728175</v>
+        <v>0.9254272384930784</v>
       </c>
       <c r="F21" t="n">
-        <v>-0.05595404036399178</v>
+        <v>0.9444796714903961</v>
       </c>
       <c r="G21" t="n">
-        <v>-0.01508135592724276</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>OCS</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>0.06256079981451537</v>
-      </c>
-      <c r="C22" t="n">
-        <v>0.3424663727403066</v>
-      </c>
-      <c r="D22" t="n">
-        <v>0.0227959297442118</v>
-      </c>
-      <c r="E22" t="n">
-        <v>-0.3232949112875109</v>
-      </c>
-      <c r="F22" t="n">
-        <v>-0.01018683624380816</v>
-      </c>
-      <c r="G22" t="n">
-        <v>-0.06030598564339989</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>Pb</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>0.2124157006893419</v>
-      </c>
-      <c r="C23" t="n">
-        <v>-0.08393313130990303</v>
-      </c>
-      <c r="D23" t="n">
-        <v>0.23298906585623</v>
-      </c>
-      <c r="E23" t="n">
-        <v>-0.06287987898983598</v>
-      </c>
-      <c r="F23" t="n">
-        <v>-0.2867597770223256</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0.08525438859070254</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>QCB</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>0.07451855749958812</v>
-      </c>
-      <c r="C24" t="n">
-        <v>0.3684464065563074</v>
-      </c>
-      <c r="D24" t="n">
-        <v>0.09341122820828777</v>
-      </c>
-      <c r="E24" t="n">
-        <v>-0.2718697253615637</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0.1857645315001332</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0.02570597526279964</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>Sb</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>-0.1723493730167432</v>
-      </c>
-      <c r="C25" t="n">
-        <v>0.2270249379889613</v>
-      </c>
-      <c r="D25" t="n">
-        <v>0.01537621960778567</v>
-      </c>
-      <c r="E25" t="n">
-        <v>0.3304007376608576</v>
-      </c>
-      <c r="F25" t="n">
-        <v>-0.08581706245394793</v>
-      </c>
-      <c r="G25" t="n">
-        <v>-0.1820909618935796</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
-        <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>0.2437986225585753</v>
-      </c>
-      <c r="C26" t="n">
-        <v>-0.07040218127850534</v>
-      </c>
-      <c r="D26" t="n">
-        <v>-0.1666206530209829</v>
-      </c>
-      <c r="E26" t="n">
-        <v>0.0369765475418331</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0.1684817118152763</v>
-      </c>
-      <c r="G26" t="n">
-        <v>-0.01537320936162412</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>Zn</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>0.2515283152383317</v>
-      </c>
-      <c r="C27" t="n">
-        <v>-0.04913556182896741</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0.09763427772862185</v>
-      </c>
-      <c r="E27" t="n">
-        <v>0.06361450815396159</v>
-      </c>
-      <c r="F27" t="n">
-        <v>-0.1976253009879765</v>
-      </c>
-      <c r="G27" t="n">
-        <v>0.1026218105241873</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>mirex</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>0.03451334187641743</v>
-      </c>
-      <c r="C28" t="n">
-        <v>-0.1110015112904317</v>
-      </c>
-      <c r="D28" t="n">
-        <v>0.3583296258781334</v>
-      </c>
-      <c r="E28" t="n">
-        <v>0.1752215647478979</v>
-      </c>
-      <c r="F28" t="n">
-        <v>0.1934098723955744</v>
-      </c>
-      <c r="G28" t="n">
-        <v>-0.1003762038932513</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>p,p'-DDD</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>0.115345875365611</v>
-      </c>
-      <c r="C29" t="n">
-        <v>-0.1550765542909818</v>
-      </c>
-      <c r="D29" t="n">
-        <v>0.3441511749737677</v>
-      </c>
-      <c r="E29" t="n">
-        <v>0.004920310326090083</v>
-      </c>
-      <c r="F29" t="n">
-        <v>0.1644809115669379</v>
-      </c>
-      <c r="G29" t="n">
-        <v>-0.205454134324473</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>p,p'-DDE</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>0.06559709252380072</v>
-      </c>
-      <c r="C30" t="n">
-        <v>-0.2257453644568954</v>
-      </c>
-      <c r="D30" t="n">
-        <v>0.3156700411816666</v>
-      </c>
-      <c r="E30" t="n">
-        <v>0.08596877451457841</v>
-      </c>
-      <c r="F30" t="n">
-        <v>0.3693856703599087</v>
-      </c>
-      <c r="G30" t="n">
-        <v>-0.2137923197285172</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="1" t="inlineStr">
-        <is>
-          <t>total PCB</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>0.1727280423566026</v>
-      </c>
-      <c r="C31" t="n">
-        <v>0.0611687594921552</v>
-      </c>
-      <c r="D31" t="n">
-        <v>0.3151799431158623</v>
-      </c>
-      <c r="E31" t="n">
-        <v>-0.06766162487470403</v>
-      </c>
-      <c r="F31" t="n">
-        <v>-0.2140701776687695</v>
-      </c>
-      <c r="G31" t="n">
-        <v>0.141928199352747</v>
+        <v>0.9589764506790596</v>
       </c>
     </row>
   </sheetData>

</xml_diff>